<commit_message>
Add usart pins for test & Modify adc and TIM configs
</commit_message>
<xml_diff>
--- a/Doc/引脚分配.xlsx
+++ b/Doc/引脚分配.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Profile\01_Projects\Personal\STM32-AutoTrace-Car\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D717F865-859F-41D4-B191-6E38C74D8E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A7A771B-98FA-41D1-95FA-06A6971C578B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{0BC2CD4C-9762-408D-8D96-6A5837F173B9}"/>
+    <workbookView xWindow="2220" yWindow="2380" windowWidth="19200" windowHeight="11170" xr2:uid="{0BC2CD4C-9762-408D-8D96-6A5837F173B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="43">
   <si>
     <t>引脚</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -174,23 +174,39 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PA0, PA1</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TIM2_CH1, CH2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PA6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>ADC1_CH6</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>PC14</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>串口调试</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PA10, PA9</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USART_RX, TX</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>串口</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PA6, PA7</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PB0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TIM3_CH1, CH2</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -606,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD03B8BF-FBCD-4097-B629-BE36F7BD0FA1}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="22.08203125" customWidth="1"/>
@@ -708,10 +724,10 @@
         <v>17</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>12</v>
@@ -743,44 +759,50 @@
     </row>
     <row r="11" spans="1:4" ht="25.5" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="25.5" customHeight="1">
-      <c r="A12" s="3" t="s">
+    <row r="13" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A13" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="25.5" customHeight="1">
-      <c r="A13" s="3"/>
-      <c r="B13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
     </row>
     <row r="14" spans="1:4" ht="25.5" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -788,7 +810,7 @@
     <row r="15" spans="1:4" ht="25.5" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -796,22 +818,30 @@
     <row r="16" spans="1:4" ht="25.5" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="2" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
     </row>
-    <row r="17" spans="1:1">
-      <c r="A17" s="1"/>
+    <row r="17" spans="1:4" ht="25.5" customHeight="1">
+      <c r="A17" s="3"/>
+      <c r="B17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="C12:C16"/>
-    <mergeCell ref="D12:D16"/>
+    <mergeCell ref="C13:C17"/>
+    <mergeCell ref="D13:D17"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="A13:A17"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>